<commit_message>
spreadsheets augmented with a few suggested values
</commit_message>
<xml_diff>
--- a/doc/crosspos/a4-deferred-crosspos.xlsx
+++ b/doc/crosspos/a4-deferred-crosspos.xlsx
@@ -13,7 +13,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1198" uniqueCount="291">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1198" uniqueCount="295">
   <si>
     <t>synset</t>
   </si>
@@ -69,6 +69,9 @@
     <t>wn:exemplifies</t>
   </si>
   <si>
+    <t>Automatisk forslag: hypernymet er en brugsmarkering, ikke et overbegreb.</t>
+  </si>
+  <si>
     <t>https://wordnet.dk/dannet/data/synset-40368</t>
   </si>
   <si>
@@ -243,6 +246,9 @@
     <t>ordklassefejl</t>
   </si>
   <si>
+    <t>Automatisk forslag: fast nominalt udtryk. Bekræft den substantiviske brug i DDO.</t>
+  </si>
+  <si>
     <t>https://wordnet.dk/dannet/data/synset-1488</t>
   </si>
   <si>
@@ -282,6 +288,9 @@
     <t>person</t>
   </si>
   <si>
+    <t>Automatisk forslag: substantiveret adjektiv (en person). Bekræft den substantiviske brug i DDO.</t>
+  </si>
+  <si>
     <t>https://wordnet.dk/dannet/data/synset-61982</t>
   </si>
   <si>
@@ -379,6 +388,9 @@
   </si>
   <si>
     <t>sprog</t>
+  </si>
+  <si>
+    <t>Automatisk forslag: substantiveret adjektiv (et sprog). Bekræft den substantiviske brug i DDO.</t>
   </si>
   <si>
     <t>https://wordnet.dk/dannet/data/synset-73502</t>
@@ -1044,18 +1056,18 @@
         <v>16</v>
       </c>
       <c r="I2" t="s" s="2">
-        <v>16</v>
+        <v>18</v>
       </c>
       <c r="J2" t="s" s="0">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="K2" t="s" s="0">
-        <v>19</v>
+        <v>20</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="s" s="1">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="B3" t="s" s="0">
         <v>12</v>
@@ -1079,18 +1091,18 @@
         <v>16</v>
       </c>
       <c r="I3" t="s" s="2">
-        <v>16</v>
+        <v>18</v>
       </c>
       <c r="J3" t="s" s="0">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="K3" t="s" s="0">
-        <v>19</v>
+        <v>20</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="s" s="1">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="B4" t="s" s="0">
         <v>12</v>
@@ -1114,18 +1126,18 @@
         <v>16</v>
       </c>
       <c r="I4" t="s" s="2">
-        <v>16</v>
+        <v>18</v>
       </c>
       <c r="J4" t="s" s="0">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="K4" t="s" s="0">
-        <v>19</v>
+        <v>20</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="s" s="1">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="B5" t="s" s="0">
         <v>12</v>
@@ -1149,18 +1161,18 @@
         <v>16</v>
       </c>
       <c r="I5" t="s" s="2">
-        <v>16</v>
+        <v>18</v>
       </c>
       <c r="J5" t="s" s="0">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="K5" t="s" s="0">
-        <v>19</v>
+        <v>20</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="s" s="1">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="B6" t="s" s="0">
         <v>12</v>
@@ -1184,18 +1196,18 @@
         <v>16</v>
       </c>
       <c r="I6" t="s" s="2">
-        <v>16</v>
+        <v>18</v>
       </c>
       <c r="J6" t="s" s="0">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="K6" t="s" s="0">
-        <v>19</v>
+        <v>20</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="s" s="1">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="B7" t="s" s="0">
         <v>12</v>
@@ -1219,18 +1231,18 @@
         <v>16</v>
       </c>
       <c r="I7" t="s" s="2">
-        <v>16</v>
+        <v>18</v>
       </c>
       <c r="J7" t="s" s="0">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="K7" t="s" s="0">
-        <v>19</v>
+        <v>20</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="s" s="1">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="B8" t="s" s="0">
         <v>12</v>
@@ -1254,18 +1266,18 @@
         <v>16</v>
       </c>
       <c r="I8" t="s" s="2">
-        <v>16</v>
+        <v>18</v>
       </c>
       <c r="J8" t="s" s="0">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="K8" t="s" s="0">
-        <v>19</v>
+        <v>20</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="s" s="1">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="B9" t="s" s="0">
         <v>12</v>
@@ -1289,18 +1301,18 @@
         <v>16</v>
       </c>
       <c r="I9" t="s" s="2">
-        <v>16</v>
+        <v>18</v>
       </c>
       <c r="J9" t="s" s="0">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="K9" t="s" s="0">
-        <v>19</v>
+        <v>20</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="s" s="1">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="B10" t="s" s="0">
         <v>12</v>
@@ -1324,18 +1336,18 @@
         <v>16</v>
       </c>
       <c r="I10" t="s" s="2">
-        <v>16</v>
+        <v>18</v>
       </c>
       <c r="J10" t="s" s="0">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="K10" t="s" s="0">
-        <v>19</v>
+        <v>20</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="s" s="1">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="B11" t="s" s="0">
         <v>12</v>
@@ -1359,18 +1371,18 @@
         <v>16</v>
       </c>
       <c r="I11" t="s" s="2">
-        <v>16</v>
+        <v>18</v>
       </c>
       <c r="J11" t="s" s="0">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="K11" t="s" s="0">
-        <v>19</v>
+        <v>20</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="s" s="1">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="B12" t="s" s="0">
         <v>12</v>
@@ -1394,18 +1406,18 @@
         <v>16</v>
       </c>
       <c r="I12" t="s" s="2">
-        <v>16</v>
+        <v>18</v>
       </c>
       <c r="J12" t="s" s="0">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="K12" t="s" s="0">
-        <v>19</v>
+        <v>20</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="s" s="1">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="B13" t="s" s="0">
         <v>12</v>
@@ -1429,18 +1441,18 @@
         <v>16</v>
       </c>
       <c r="I13" t="s" s="2">
-        <v>16</v>
+        <v>18</v>
       </c>
       <c r="J13" t="s" s="0">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="K13" t="s" s="0">
-        <v>19</v>
+        <v>20</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="s" s="1">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="B14" t="s" s="0">
         <v>12</v>
@@ -1464,18 +1476,18 @@
         <v>16</v>
       </c>
       <c r="I14" t="s" s="2">
-        <v>16</v>
+        <v>18</v>
       </c>
       <c r="J14" t="s" s="0">
-        <v>43</v>
+        <v>44</v>
       </c>
       <c r="K14" t="s" s="0">
-        <v>19</v>
+        <v>20</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="s" s="1">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="B15" t="s" s="0">
         <v>12</v>
@@ -1499,18 +1511,18 @@
         <v>16</v>
       </c>
       <c r="I15" t="s" s="2">
-        <v>16</v>
+        <v>18</v>
       </c>
       <c r="J15" t="s" s="0">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="K15" t="s" s="0">
-        <v>19</v>
+        <v>20</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="s" s="1">
-        <v>46</v>
+        <v>47</v>
       </c>
       <c r="B16" t="s" s="0">
         <v>12</v>
@@ -1534,18 +1546,18 @@
         <v>16</v>
       </c>
       <c r="I16" t="s" s="2">
-        <v>16</v>
+        <v>18</v>
       </c>
       <c r="J16" t="s" s="0">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="K16" t="s" s="0">
-        <v>19</v>
+        <v>20</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="s" s="1">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="B17" t="s" s="0">
         <v>12</v>
@@ -1569,18 +1581,18 @@
         <v>16</v>
       </c>
       <c r="I17" t="s" s="2">
-        <v>16</v>
+        <v>18</v>
       </c>
       <c r="J17" t="s" s="0">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="K17" t="s" s="0">
-        <v>19</v>
+        <v>20</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="s" s="1">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="B18" t="s" s="0">
         <v>12</v>
@@ -1604,18 +1616,18 @@
         <v>16</v>
       </c>
       <c r="I18" t="s" s="2">
-        <v>16</v>
+        <v>18</v>
       </c>
       <c r="J18" t="s" s="0">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="K18" t="s" s="0">
-        <v>19</v>
+        <v>20</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="s" s="1">
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="B19" t="s" s="0">
         <v>12</v>
@@ -1639,18 +1651,18 @@
         <v>16</v>
       </c>
       <c r="I19" t="s" s="2">
-        <v>16</v>
+        <v>18</v>
       </c>
       <c r="J19" t="s" s="0">
-        <v>53</v>
+        <v>54</v>
       </c>
       <c r="K19" t="s" s="0">
-        <v>19</v>
+        <v>20</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="s" s="1">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="B20" t="s" s="0">
         <v>12</v>
@@ -1674,18 +1686,18 @@
         <v>16</v>
       </c>
       <c r="I20" t="s" s="2">
-        <v>16</v>
+        <v>18</v>
       </c>
       <c r="J20" t="s" s="0">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="K20" t="s" s="0">
-        <v>19</v>
+        <v>20</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="s" s="1">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="B21" t="s" s="0">
         <v>12</v>
@@ -1709,18 +1721,18 @@
         <v>16</v>
       </c>
       <c r="I21" t="s" s="2">
-        <v>16</v>
+        <v>18</v>
       </c>
       <c r="J21" t="s" s="0">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="K21" t="s" s="0">
-        <v>19</v>
+        <v>20</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="s" s="1">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="B22" t="s" s="0">
         <v>12</v>
@@ -1744,18 +1756,18 @@
         <v>16</v>
       </c>
       <c r="I22" t="s" s="2">
-        <v>16</v>
+        <v>18</v>
       </c>
       <c r="J22" t="s" s="0">
-        <v>59</v>
+        <v>60</v>
       </c>
       <c r="K22" t="s" s="0">
-        <v>19</v>
+        <v>20</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="s" s="1">
-        <v>60</v>
+        <v>61</v>
       </c>
       <c r="B23" t="s" s="0">
         <v>12</v>
@@ -1779,18 +1791,18 @@
         <v>16</v>
       </c>
       <c r="I23" t="s" s="2">
-        <v>16</v>
+        <v>18</v>
       </c>
       <c r="J23" t="s" s="0">
-        <v>61</v>
+        <v>62</v>
       </c>
       <c r="K23" t="s" s="0">
-        <v>19</v>
+        <v>20</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="s" s="1">
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="B24" t="s" s="0">
         <v>12</v>
@@ -1814,18 +1826,18 @@
         <v>16</v>
       </c>
       <c r="I24" t="s" s="2">
-        <v>16</v>
+        <v>18</v>
       </c>
       <c r="J24" t="s" s="0">
-        <v>63</v>
+        <v>64</v>
       </c>
       <c r="K24" t="s" s="0">
-        <v>19</v>
+        <v>20</v>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="s" s="1">
-        <v>64</v>
+        <v>65</v>
       </c>
       <c r="B25" t="s" s="0">
         <v>12</v>
@@ -1849,18 +1861,18 @@
         <v>16</v>
       </c>
       <c r="I25" t="s" s="2">
-        <v>16</v>
+        <v>18</v>
       </c>
       <c r="J25" t="s" s="0">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="K25" t="s" s="0">
-        <v>19</v>
+        <v>20</v>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="s" s="1">
-        <v>66</v>
+        <v>67</v>
       </c>
       <c r="B26" t="s" s="0">
         <v>12</v>
@@ -1884,24 +1896,24 @@
         <v>16</v>
       </c>
       <c r="I26" t="s" s="2">
-        <v>16</v>
+        <v>18</v>
       </c>
       <c r="J26" t="s" s="0">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="K26" t="s" s="0">
-        <v>19</v>
+        <v>20</v>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="s" s="1">
-        <v>68</v>
+        <v>69</v>
       </c>
       <c r="B27" t="s" s="0">
         <v>12</v>
       </c>
       <c r="C27" t="s" s="1">
-        <v>69</v>
+        <v>70</v>
       </c>
       <c r="D27" t="s" s="0">
         <v>14</v>
@@ -1919,30 +1931,30 @@
         <v>16</v>
       </c>
       <c r="I27" t="s" s="2">
-        <v>16</v>
+        <v>18</v>
       </c>
       <c r="J27" t="s" s="0">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="K27" t="s" s="0">
-        <v>71</v>
+        <v>72</v>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="s" s="1">
-        <v>72</v>
+        <v>73</v>
       </c>
       <c r="B28" t="s" s="0">
         <v>12</v>
       </c>
       <c r="C28" t="s" s="1">
-        <v>73</v>
+        <v>74</v>
       </c>
       <c r="D28" t="s" s="0">
-        <v>74</v>
+        <v>75</v>
       </c>
       <c r="E28" t="s" s="0">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="F28" t="s" s="2">
         <v>16</v>
@@ -1954,30 +1966,30 @@
         <v>16</v>
       </c>
       <c r="I28" t="s" s="2">
-        <v>16</v>
+        <v>77</v>
       </c>
       <c r="J28" t="s" s="0">
-        <v>76</v>
+        <v>78</v>
       </c>
       <c r="K28" t="s" s="0">
-        <v>77</v>
+        <v>79</v>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="s" s="1">
-        <v>78</v>
+        <v>80</v>
       </c>
       <c r="B29" t="s" s="0">
         <v>12</v>
       </c>
       <c r="C29" t="s" s="1">
-        <v>79</v>
+        <v>81</v>
       </c>
       <c r="D29" t="s" s="0">
-        <v>74</v>
+        <v>75</v>
       </c>
       <c r="E29" t="s" s="0">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="F29" t="s" s="2">
         <v>16</v>
@@ -1989,30 +2001,30 @@
         <v>16</v>
       </c>
       <c r="I29" t="s" s="2">
-        <v>16</v>
+        <v>77</v>
       </c>
       <c r="J29" t="s" s="0">
-        <v>80</v>
+        <v>82</v>
       </c>
       <c r="K29" t="s" s="0">
-        <v>81</v>
+        <v>83</v>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="s" s="1">
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="B30" t="s" s="0">
         <v>12</v>
       </c>
       <c r="C30" t="s" s="1">
-        <v>83</v>
+        <v>85</v>
       </c>
       <c r="D30" t="s" s="0">
-        <v>74</v>
+        <v>75</v>
       </c>
       <c r="E30" t="s" s="0">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="F30" t="s" s="2">
         <v>16</v>
@@ -2024,30 +2036,30 @@
         <v>16</v>
       </c>
       <c r="I30" t="s" s="2">
-        <v>16</v>
+        <v>77</v>
       </c>
       <c r="J30" t="s" s="0">
-        <v>84</v>
+        <v>86</v>
       </c>
       <c r="K30" t="s" s="0">
-        <v>85</v>
+        <v>87</v>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="s" s="1">
-        <v>86</v>
+        <v>88</v>
       </c>
       <c r="B31" t="s" s="0">
         <v>12</v>
       </c>
       <c r="C31" t="s" s="1">
-        <v>87</v>
+        <v>89</v>
       </c>
       <c r="D31" t="s" s="0">
-        <v>88</v>
+        <v>90</v>
       </c>
       <c r="E31" t="s" s="0">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="F31" t="s" s="2">
         <v>16</v>
@@ -2059,100 +2071,100 @@
         <v>16</v>
       </c>
       <c r="I31" t="s" s="2">
-        <v>16</v>
+        <v>91</v>
       </c>
       <c r="J31" t="s" s="0">
-        <v>89</v>
+        <v>92</v>
       </c>
       <c r="K31" t="s" s="0">
-        <v>90</v>
+        <v>93</v>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="s" s="1">
+        <v>94</v>
+      </c>
+      <c r="B32" t="s" s="0">
+        <v>12</v>
+      </c>
+      <c r="C32" t="s" s="1">
+        <v>89</v>
+      </c>
+      <c r="D32" t="s" s="0">
+        <v>90</v>
+      </c>
+      <c r="E32" t="s" s="0">
+        <v>76</v>
+      </c>
+      <c r="F32" t="s" s="2">
+        <v>16</v>
+      </c>
+      <c r="G32" t="s" s="2">
+        <v>16</v>
+      </c>
+      <c r="H32" t="s" s="2">
+        <v>16</v>
+      </c>
+      <c r="I32" t="s" s="2">
         <v>91</v>
       </c>
-      <c r="B32" t="s" s="0">
-        <v>12</v>
-      </c>
-      <c r="C32" t="s" s="1">
-        <v>87</v>
-      </c>
-      <c r="D32" t="s" s="0">
-        <v>88</v>
-      </c>
-      <c r="E32" t="s" s="0">
-        <v>75</v>
-      </c>
-      <c r="F32" t="s" s="2">
-        <v>16</v>
-      </c>
-      <c r="G32" t="s" s="2">
-        <v>16</v>
-      </c>
-      <c r="H32" t="s" s="2">
-        <v>16</v>
-      </c>
-      <c r="I32" t="s" s="2">
-        <v>16</v>
-      </c>
       <c r="J32" t="s" s="0">
-        <v>92</v>
+        <v>95</v>
       </c>
       <c r="K32" t="s" s="0">
-        <v>90</v>
+        <v>93</v>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="s" s="1">
+        <v>96</v>
+      </c>
+      <c r="B33" t="s" s="0">
+        <v>12</v>
+      </c>
+      <c r="C33" t="s" s="1">
+        <v>89</v>
+      </c>
+      <c r="D33" t="s" s="0">
+        <v>90</v>
+      </c>
+      <c r="E33" t="s" s="0">
+        <v>76</v>
+      </c>
+      <c r="F33" t="s" s="2">
+        <v>16</v>
+      </c>
+      <c r="G33" t="s" s="2">
+        <v>16</v>
+      </c>
+      <c r="H33" t="s" s="2">
+        <v>16</v>
+      </c>
+      <c r="I33" t="s" s="2">
+        <v>91</v>
+      </c>
+      <c r="J33" t="s" s="0">
+        <v>97</v>
+      </c>
+      <c r="K33" t="s" s="0">
         <v>93</v>
-      </c>
-      <c r="B33" t="s" s="0">
-        <v>12</v>
-      </c>
-      <c r="C33" t="s" s="1">
-        <v>87</v>
-      </c>
-      <c r="D33" t="s" s="0">
-        <v>88</v>
-      </c>
-      <c r="E33" t="s" s="0">
-        <v>75</v>
-      </c>
-      <c r="F33" t="s" s="2">
-        <v>16</v>
-      </c>
-      <c r="G33" t="s" s="2">
-        <v>16</v>
-      </c>
-      <c r="H33" t="s" s="2">
-        <v>16</v>
-      </c>
-      <c r="I33" t="s" s="2">
-        <v>16</v>
-      </c>
-      <c r="J33" t="s" s="0">
-        <v>94</v>
-      </c>
-      <c r="K33" t="s" s="0">
-        <v>90</v>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="s" s="1">
-        <v>95</v>
+        <v>98</v>
       </c>
       <c r="B34" t="s" s="0">
         <v>12</v>
       </c>
       <c r="C34" t="s" s="1">
-        <v>87</v>
+        <v>89</v>
       </c>
       <c r="D34" t="s" s="0">
-        <v>88</v>
+        <v>90</v>
       </c>
       <c r="E34" t="s" s="0">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="F34" t="s" s="2">
         <v>16</v>
@@ -2164,30 +2176,30 @@
         <v>16</v>
       </c>
       <c r="I34" t="s" s="2">
-        <v>16</v>
+        <v>91</v>
       </c>
       <c r="J34" t="s" s="0">
-        <v>96</v>
+        <v>99</v>
       </c>
       <c r="K34" t="s" s="0">
-        <v>90</v>
+        <v>93</v>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="s" s="1">
-        <v>97</v>
+        <v>100</v>
       </c>
       <c r="B35" t="s" s="0">
         <v>12</v>
       </c>
       <c r="C35" t="s" s="1">
-        <v>87</v>
+        <v>89</v>
       </c>
       <c r="D35" t="s" s="0">
-        <v>88</v>
+        <v>90</v>
       </c>
       <c r="E35" t="s" s="0">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="F35" t="s" s="2">
         <v>16</v>
@@ -2199,30 +2211,30 @@
         <v>16</v>
       </c>
       <c r="I35" t="s" s="2">
-        <v>16</v>
+        <v>91</v>
       </c>
       <c r="J35" t="s" s="0">
-        <v>98</v>
+        <v>101</v>
       </c>
       <c r="K35" t="s" s="0">
-        <v>90</v>
+        <v>93</v>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="s" s="1">
-        <v>99</v>
+        <v>102</v>
       </c>
       <c r="B36" t="s" s="0">
         <v>12</v>
       </c>
       <c r="C36" t="s" s="1">
-        <v>87</v>
+        <v>89</v>
       </c>
       <c r="D36" t="s" s="0">
-        <v>88</v>
+        <v>90</v>
       </c>
       <c r="E36" t="s" s="0">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="F36" t="s" s="2">
         <v>16</v>
@@ -2234,30 +2246,30 @@
         <v>16</v>
       </c>
       <c r="I36" t="s" s="2">
-        <v>16</v>
+        <v>91</v>
       </c>
       <c r="J36" t="s" s="0">
-        <v>100</v>
+        <v>103</v>
       </c>
       <c r="K36" t="s" s="0">
-        <v>90</v>
+        <v>93</v>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="s" s="1">
-        <v>101</v>
+        <v>104</v>
       </c>
       <c r="B37" t="s" s="0">
         <v>12</v>
       </c>
       <c r="C37" t="s" s="1">
-        <v>102</v>
+        <v>105</v>
       </c>
       <c r="D37" t="s" s="0">
-        <v>88</v>
+        <v>90</v>
       </c>
       <c r="E37" t="s" s="0">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="F37" t="s" s="2">
         <v>16</v>
@@ -2269,30 +2281,30 @@
         <v>16</v>
       </c>
       <c r="I37" t="s" s="2">
-        <v>16</v>
+        <v>91</v>
       </c>
       <c r="J37" t="s" s="0">
-        <v>103</v>
+        <v>106</v>
       </c>
       <c r="K37" t="s" s="0">
-        <v>104</v>
+        <v>107</v>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="s" s="1">
+        <v>108</v>
+      </c>
+      <c r="B38" t="s" s="0">
+        <v>12</v>
+      </c>
+      <c r="C38" t="s" s="1">
         <v>105</v>
       </c>
-      <c r="B38" t="s" s="0">
-        <v>12</v>
-      </c>
-      <c r="C38" t="s" s="1">
-        <v>102</v>
-      </c>
       <c r="D38" t="s" s="0">
-        <v>88</v>
+        <v>90</v>
       </c>
       <c r="E38" t="s" s="0">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="F38" t="s" s="2">
         <v>16</v>
@@ -2304,65 +2316,65 @@
         <v>16</v>
       </c>
       <c r="I38" t="s" s="2">
-        <v>16</v>
+        <v>91</v>
       </c>
       <c r="J38" t="s" s="0">
-        <v>106</v>
+        <v>109</v>
       </c>
       <c r="K38" t="s" s="0">
-        <v>104</v>
+        <v>107</v>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="s" s="1">
+        <v>110</v>
+      </c>
+      <c r="B39" t="s" s="0">
+        <v>12</v>
+      </c>
+      <c r="C39" t="s" s="1">
+        <v>105</v>
+      </c>
+      <c r="D39" t="s" s="0">
+        <v>90</v>
+      </c>
+      <c r="E39" t="s" s="0">
+        <v>76</v>
+      </c>
+      <c r="F39" t="s" s="2">
+        <v>16</v>
+      </c>
+      <c r="G39" t="s" s="2">
+        <v>16</v>
+      </c>
+      <c r="H39" t="s" s="2">
+        <v>16</v>
+      </c>
+      <c r="I39" t="s" s="2">
+        <v>91</v>
+      </c>
+      <c r="J39" t="s" s="0">
+        <v>111</v>
+      </c>
+      <c r="K39" t="s" s="0">
         <v>107</v>
-      </c>
-      <c r="B39" t="s" s="0">
-        <v>12</v>
-      </c>
-      <c r="C39" t="s" s="1">
-        <v>102</v>
-      </c>
-      <c r="D39" t="s" s="0">
-        <v>88</v>
-      </c>
-      <c r="E39" t="s" s="0">
-        <v>75</v>
-      </c>
-      <c r="F39" t="s" s="2">
-        <v>16</v>
-      </c>
-      <c r="G39" t="s" s="2">
-        <v>16</v>
-      </c>
-      <c r="H39" t="s" s="2">
-        <v>16</v>
-      </c>
-      <c r="I39" t="s" s="2">
-        <v>16</v>
-      </c>
-      <c r="J39" t="s" s="0">
-        <v>108</v>
-      </c>
-      <c r="K39" t="s" s="0">
-        <v>104</v>
       </c>
     </row>
     <row r="40">
       <c r="A40" t="s" s="1">
-        <v>109</v>
+        <v>112</v>
       </c>
       <c r="B40" t="s" s="0">
         <v>12</v>
       </c>
       <c r="C40" t="s" s="1">
-        <v>102</v>
+        <v>105</v>
       </c>
       <c r="D40" t="s" s="0">
-        <v>88</v>
+        <v>90</v>
       </c>
       <c r="E40" t="s" s="0">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="F40" t="s" s="2">
         <v>16</v>
@@ -2374,30 +2386,30 @@
         <v>16</v>
       </c>
       <c r="I40" t="s" s="2">
-        <v>16</v>
+        <v>91</v>
       </c>
       <c r="J40" t="s" s="0">
-        <v>110</v>
+        <v>113</v>
       </c>
       <c r="K40" t="s" s="0">
-        <v>104</v>
+        <v>107</v>
       </c>
     </row>
     <row r="41">
       <c r="A41" t="s" s="1">
-        <v>111</v>
+        <v>114</v>
       </c>
       <c r="B41" t="s" s="0">
         <v>12</v>
       </c>
       <c r="C41" t="s" s="1">
-        <v>102</v>
+        <v>105</v>
       </c>
       <c r="D41" t="s" s="0">
-        <v>88</v>
+        <v>90</v>
       </c>
       <c r="E41" t="s" s="0">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="F41" t="s" s="2">
         <v>16</v>
@@ -2409,30 +2421,30 @@
         <v>16</v>
       </c>
       <c r="I41" t="s" s="2">
-        <v>16</v>
+        <v>91</v>
       </c>
       <c r="J41" t="s" s="0">
-        <v>112</v>
+        <v>115</v>
       </c>
       <c r="K41" t="s" s="0">
-        <v>104</v>
+        <v>107</v>
       </c>
     </row>
     <row r="42">
       <c r="A42" t="s" s="1">
-        <v>113</v>
+        <v>116</v>
       </c>
       <c r="B42" t="s" s="0">
         <v>12</v>
       </c>
       <c r="C42" t="s" s="1">
-        <v>102</v>
+        <v>105</v>
       </c>
       <c r="D42" t="s" s="0">
-        <v>88</v>
+        <v>90</v>
       </c>
       <c r="E42" t="s" s="0">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="F42" t="s" s="2">
         <v>16</v>
@@ -2444,30 +2456,30 @@
         <v>16</v>
       </c>
       <c r="I42" t="s" s="2">
-        <v>16</v>
+        <v>91</v>
       </c>
       <c r="J42" t="s" s="0">
-        <v>114</v>
+        <v>117</v>
       </c>
       <c r="K42" t="s" s="0">
-        <v>104</v>
+        <v>107</v>
       </c>
     </row>
     <row r="43">
       <c r="A43" t="s" s="1">
-        <v>115</v>
+        <v>118</v>
       </c>
       <c r="B43" t="s" s="0">
         <v>12</v>
       </c>
       <c r="C43" t="s" s="1">
-        <v>116</v>
+        <v>119</v>
       </c>
       <c r="D43" t="s" s="0">
-        <v>88</v>
+        <v>90</v>
       </c>
       <c r="E43" t="s" s="0">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="F43" t="s" s="2">
         <v>16</v>
@@ -2479,30 +2491,30 @@
         <v>16</v>
       </c>
       <c r="I43" t="s" s="2">
-        <v>16</v>
+        <v>91</v>
       </c>
       <c r="J43" t="s" s="0">
-        <v>117</v>
+        <v>120</v>
       </c>
       <c r="K43" t="s" s="0">
-        <v>118</v>
+        <v>121</v>
       </c>
     </row>
     <row r="44">
       <c r="A44" t="s" s="1">
-        <v>119</v>
+        <v>122</v>
       </c>
       <c r="B44" t="s" s="0">
         <v>12</v>
       </c>
       <c r="C44" t="s" s="1">
-        <v>120</v>
+        <v>123</v>
       </c>
       <c r="D44" t="s" s="0">
-        <v>121</v>
+        <v>124</v>
       </c>
       <c r="E44" t="s" s="0">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="F44" t="s" s="2">
         <v>16</v>
@@ -2514,30 +2526,30 @@
         <v>16</v>
       </c>
       <c r="I44" t="s" s="2">
-        <v>16</v>
+        <v>125</v>
       </c>
       <c r="J44" t="s" s="0">
-        <v>122</v>
+        <v>126</v>
       </c>
       <c r="K44" t="s" s="0">
-        <v>123</v>
+        <v>127</v>
       </c>
     </row>
     <row r="45">
       <c r="A45" t="s" s="1">
-        <v>124</v>
+        <v>128</v>
       </c>
       <c r="B45" t="s" s="0">
         <v>12</v>
       </c>
       <c r="C45" t="s" s="1">
-        <v>120</v>
+        <v>123</v>
       </c>
       <c r="D45" t="s" s="0">
-        <v>121</v>
+        <v>124</v>
       </c>
       <c r="E45" t="s" s="0">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="F45" t="s" s="2">
         <v>16</v>
@@ -2549,30 +2561,30 @@
         <v>16</v>
       </c>
       <c r="I45" t="s" s="2">
-        <v>16</v>
+        <v>125</v>
       </c>
       <c r="J45" t="s" s="0">
-        <v>125</v>
+        <v>129</v>
       </c>
       <c r="K45" t="s" s="0">
-        <v>123</v>
+        <v>127</v>
       </c>
     </row>
     <row r="46">
       <c r="A46" t="s" s="1">
-        <v>126</v>
+        <v>130</v>
       </c>
       <c r="B46" t="s" s="0">
         <v>12</v>
       </c>
       <c r="C46" t="s" s="1">
-        <v>120</v>
+        <v>123</v>
       </c>
       <c r="D46" t="s" s="0">
-        <v>121</v>
+        <v>124</v>
       </c>
       <c r="E46" t="s" s="0">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="F46" t="s" s="2">
         <v>16</v>
@@ -2584,30 +2596,30 @@
         <v>16</v>
       </c>
       <c r="I46" t="s" s="2">
-        <v>16</v>
+        <v>125</v>
       </c>
       <c r="J46" t="s" s="0">
+        <v>131</v>
+      </c>
+      <c r="K46" t="s" s="0">
         <v>127</v>
-      </c>
-      <c r="K46" t="s" s="0">
-        <v>123</v>
       </c>
     </row>
     <row r="47">
       <c r="A47" t="s" s="1">
-        <v>128</v>
+        <v>132</v>
       </c>
       <c r="B47" t="s" s="0">
         <v>12</v>
       </c>
       <c r="C47" t="s" s="1">
-        <v>129</v>
+        <v>133</v>
       </c>
       <c r="D47" t="s" s="0">
-        <v>121</v>
+        <v>124</v>
       </c>
       <c r="E47" t="s" s="0">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="F47" t="s" s="2">
         <v>16</v>
@@ -2619,30 +2631,30 @@
         <v>16</v>
       </c>
       <c r="I47" t="s" s="2">
-        <v>16</v>
+        <v>125</v>
       </c>
       <c r="J47" t="s" s="0">
-        <v>130</v>
+        <v>134</v>
       </c>
       <c r="K47" t="s" s="0">
-        <v>131</v>
+        <v>135</v>
       </c>
     </row>
     <row r="48">
       <c r="A48" t="s" s="1">
-        <v>132</v>
+        <v>136</v>
       </c>
       <c r="B48" t="s" s="0">
         <v>12</v>
       </c>
       <c r="C48" t="s" s="1">
-        <v>129</v>
+        <v>133</v>
       </c>
       <c r="D48" t="s" s="0">
-        <v>121</v>
+        <v>124</v>
       </c>
       <c r="E48" t="s" s="0">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="F48" t="s" s="2">
         <v>16</v>
@@ -2654,30 +2666,30 @@
         <v>16</v>
       </c>
       <c r="I48" t="s" s="2">
-        <v>16</v>
+        <v>125</v>
       </c>
       <c r="J48" t="s" s="0">
-        <v>133</v>
+        <v>137</v>
       </c>
       <c r="K48" t="s" s="0">
-        <v>131</v>
+        <v>135</v>
       </c>
     </row>
     <row r="49">
       <c r="A49" t="s" s="1">
-        <v>134</v>
+        <v>138</v>
       </c>
       <c r="B49" t="s" s="0">
         <v>12</v>
       </c>
       <c r="C49" t="s" s="1">
-        <v>129</v>
+        <v>133</v>
       </c>
       <c r="D49" t="s" s="0">
-        <v>121</v>
+        <v>124</v>
       </c>
       <c r="E49" t="s" s="0">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="F49" t="s" s="2">
         <v>16</v>
@@ -2689,30 +2701,30 @@
         <v>16</v>
       </c>
       <c r="I49" t="s" s="2">
-        <v>16</v>
+        <v>125</v>
       </c>
       <c r="J49" t="s" s="0">
+        <v>139</v>
+      </c>
+      <c r="K49" t="s" s="0">
         <v>135</v>
-      </c>
-      <c r="K49" t="s" s="0">
-        <v>131</v>
       </c>
     </row>
     <row r="50">
       <c r="A50" t="s" s="1">
-        <v>136</v>
+        <v>140</v>
       </c>
       <c r="B50" t="s" s="0">
         <v>12</v>
       </c>
       <c r="C50" t="s" s="1">
-        <v>129</v>
+        <v>133</v>
       </c>
       <c r="D50" t="s" s="0">
-        <v>121</v>
+        <v>124</v>
       </c>
       <c r="E50" t="s" s="0">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="F50" t="s" s="2">
         <v>16</v>
@@ -2724,30 +2736,30 @@
         <v>16</v>
       </c>
       <c r="I50" t="s" s="2">
-        <v>16</v>
+        <v>125</v>
       </c>
       <c r="J50" t="s" s="0">
-        <v>137</v>
+        <v>141</v>
       </c>
       <c r="K50" t="s" s="0">
-        <v>131</v>
+        <v>135</v>
       </c>
     </row>
     <row r="51">
       <c r="A51" t="s" s="1">
-        <v>138</v>
+        <v>142</v>
       </c>
       <c r="B51" t="s" s="0">
         <v>12</v>
       </c>
       <c r="C51" t="s" s="1">
-        <v>129</v>
+        <v>133</v>
       </c>
       <c r="D51" t="s" s="0">
-        <v>121</v>
+        <v>124</v>
       </c>
       <c r="E51" t="s" s="0">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="F51" t="s" s="2">
         <v>16</v>
@@ -2759,30 +2771,30 @@
         <v>16</v>
       </c>
       <c r="I51" t="s" s="2">
-        <v>16</v>
+        <v>125</v>
       </c>
       <c r="J51" t="s" s="0">
-        <v>139</v>
+        <v>143</v>
       </c>
       <c r="K51" t="s" s="0">
-        <v>131</v>
+        <v>135</v>
       </c>
     </row>
     <row r="52">
       <c r="A52" t="s" s="1">
-        <v>140</v>
+        <v>144</v>
       </c>
       <c r="B52" t="s" s="0">
         <v>12</v>
       </c>
       <c r="C52" t="s" s="1">
-        <v>129</v>
+        <v>133</v>
       </c>
       <c r="D52" t="s" s="0">
-        <v>121</v>
+        <v>124</v>
       </c>
       <c r="E52" t="s" s="0">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="F52" t="s" s="2">
         <v>16</v>
@@ -2794,30 +2806,30 @@
         <v>16</v>
       </c>
       <c r="I52" t="s" s="2">
-        <v>16</v>
+        <v>125</v>
       </c>
       <c r="J52" t="s" s="0">
-        <v>141</v>
+        <v>145</v>
       </c>
       <c r="K52" t="s" s="0">
-        <v>131</v>
+        <v>135</v>
       </c>
     </row>
     <row r="53">
       <c r="A53" t="s" s="1">
-        <v>142</v>
+        <v>146</v>
       </c>
       <c r="B53" t="s" s="0">
         <v>12</v>
       </c>
       <c r="C53" t="s" s="1">
-        <v>129</v>
+        <v>133</v>
       </c>
       <c r="D53" t="s" s="0">
-        <v>121</v>
+        <v>124</v>
       </c>
       <c r="E53" t="s" s="0">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="F53" t="s" s="2">
         <v>16</v>
@@ -2829,30 +2841,30 @@
         <v>16</v>
       </c>
       <c r="I53" t="s" s="2">
-        <v>16</v>
+        <v>125</v>
       </c>
       <c r="J53" t="s" s="0">
-        <v>143</v>
+        <v>147</v>
       </c>
       <c r="K53" t="s" s="0">
-        <v>131</v>
+        <v>135</v>
       </c>
     </row>
     <row r="54">
       <c r="A54" t="s" s="1">
-        <v>144</v>
+        <v>148</v>
       </c>
       <c r="B54" t="s" s="0">
         <v>12</v>
       </c>
       <c r="C54" t="s" s="1">
-        <v>129</v>
+        <v>133</v>
       </c>
       <c r="D54" t="s" s="0">
-        <v>121</v>
+        <v>124</v>
       </c>
       <c r="E54" t="s" s="0">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="F54" t="s" s="2">
         <v>16</v>
@@ -2864,30 +2876,30 @@
         <v>16</v>
       </c>
       <c r="I54" t="s" s="2">
-        <v>16</v>
+        <v>125</v>
       </c>
       <c r="J54" t="s" s="0">
-        <v>145</v>
+        <v>149</v>
       </c>
       <c r="K54" t="s" s="0">
-        <v>131</v>
+        <v>135</v>
       </c>
     </row>
     <row r="55">
       <c r="A55" t="s" s="1">
-        <v>146</v>
+        <v>150</v>
       </c>
       <c r="B55" t="s" s="0">
         <v>12</v>
       </c>
       <c r="C55" t="s" s="1">
-        <v>129</v>
+        <v>133</v>
       </c>
       <c r="D55" t="s" s="0">
-        <v>121</v>
+        <v>124</v>
       </c>
       <c r="E55" t="s" s="0">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="F55" t="s" s="2">
         <v>16</v>
@@ -2899,30 +2911,30 @@
         <v>16</v>
       </c>
       <c r="I55" t="s" s="2">
-        <v>16</v>
+        <v>125</v>
       </c>
       <c r="J55" t="s" s="0">
-        <v>147</v>
+        <v>151</v>
       </c>
       <c r="K55" t="s" s="0">
-        <v>131</v>
+        <v>135</v>
       </c>
     </row>
     <row r="56">
       <c r="A56" t="s" s="1">
-        <v>148</v>
+        <v>152</v>
       </c>
       <c r="B56" t="s" s="0">
         <v>12</v>
       </c>
       <c r="C56" t="s" s="1">
-        <v>129</v>
+        <v>133</v>
       </c>
       <c r="D56" t="s" s="0">
-        <v>121</v>
+        <v>124</v>
       </c>
       <c r="E56" t="s" s="0">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="F56" t="s" s="2">
         <v>16</v>
@@ -2934,30 +2946,30 @@
         <v>16</v>
       </c>
       <c r="I56" t="s" s="2">
-        <v>16</v>
+        <v>125</v>
       </c>
       <c r="J56" t="s" s="0">
-        <v>149</v>
+        <v>153</v>
       </c>
       <c r="K56" t="s" s="0">
-        <v>131</v>
+        <v>135</v>
       </c>
     </row>
     <row r="57">
       <c r="A57" t="s" s="1">
-        <v>150</v>
+        <v>154</v>
       </c>
       <c r="B57" t="s" s="0">
         <v>12</v>
       </c>
       <c r="C57" t="s" s="1">
-        <v>129</v>
+        <v>133</v>
       </c>
       <c r="D57" t="s" s="0">
-        <v>121</v>
+        <v>124</v>
       </c>
       <c r="E57" t="s" s="0">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="F57" t="s" s="2">
         <v>16</v>
@@ -2969,30 +2981,30 @@
         <v>16</v>
       </c>
       <c r="I57" t="s" s="2">
-        <v>16</v>
+        <v>125</v>
       </c>
       <c r="J57" t="s" s="0">
-        <v>151</v>
+        <v>155</v>
       </c>
       <c r="K57" t="s" s="0">
-        <v>131</v>
+        <v>135</v>
       </c>
     </row>
     <row r="58">
       <c r="A58" t="s" s="1">
-        <v>152</v>
+        <v>156</v>
       </c>
       <c r="B58" t="s" s="0">
         <v>12</v>
       </c>
       <c r="C58" t="s" s="1">
-        <v>153</v>
+        <v>157</v>
       </c>
       <c r="D58" t="s" s="0">
-        <v>121</v>
+        <v>124</v>
       </c>
       <c r="E58" t="s" s="0">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="F58" t="s" s="2">
         <v>16</v>
@@ -3004,30 +3016,30 @@
         <v>16</v>
       </c>
       <c r="I58" t="s" s="2">
-        <v>16</v>
+        <v>125</v>
       </c>
       <c r="J58" t="s" s="0">
-        <v>154</v>
+        <v>158</v>
       </c>
       <c r="K58" t="s" s="0">
-        <v>155</v>
+        <v>159</v>
       </c>
     </row>
     <row r="59">
       <c r="A59" t="s" s="1">
-        <v>156</v>
+        <v>160</v>
       </c>
       <c r="B59" t="s" s="0">
         <v>12</v>
       </c>
       <c r="C59" t="s" s="1">
-        <v>153</v>
+        <v>157</v>
       </c>
       <c r="D59" t="s" s="0">
-        <v>121</v>
+        <v>124</v>
       </c>
       <c r="E59" t="s" s="0">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="F59" t="s" s="2">
         <v>16</v>
@@ -3039,30 +3051,30 @@
         <v>16</v>
       </c>
       <c r="I59" t="s" s="2">
-        <v>16</v>
+        <v>125</v>
       </c>
       <c r="J59" t="s" s="0">
-        <v>157</v>
+        <v>161</v>
       </c>
       <c r="K59" t="s" s="0">
-        <v>155</v>
+        <v>159</v>
       </c>
     </row>
     <row r="60">
       <c r="A60" t="s" s="1">
-        <v>158</v>
+        <v>162</v>
       </c>
       <c r="B60" t="s" s="0">
         <v>12</v>
       </c>
       <c r="C60" t="s" s="1">
-        <v>153</v>
+        <v>157</v>
       </c>
       <c r="D60" t="s" s="0">
-        <v>121</v>
+        <v>124</v>
       </c>
       <c r="E60" t="s" s="0">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="F60" t="s" s="2">
         <v>16</v>
@@ -3074,30 +3086,30 @@
         <v>16</v>
       </c>
       <c r="I60" t="s" s="2">
-        <v>16</v>
+        <v>125</v>
       </c>
       <c r="J60" t="s" s="0">
+        <v>163</v>
+      </c>
+      <c r="K60" t="s" s="0">
         <v>159</v>
-      </c>
-      <c r="K60" t="s" s="0">
-        <v>155</v>
       </c>
     </row>
     <row r="61">
       <c r="A61" t="s" s="1">
-        <v>160</v>
+        <v>164</v>
       </c>
       <c r="B61" t="s" s="0">
         <v>12</v>
       </c>
       <c r="C61" t="s" s="1">
-        <v>153</v>
+        <v>157</v>
       </c>
       <c r="D61" t="s" s="0">
-        <v>121</v>
+        <v>124</v>
       </c>
       <c r="E61" t="s" s="0">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="F61" t="s" s="2">
         <v>16</v>
@@ -3109,30 +3121,30 @@
         <v>16</v>
       </c>
       <c r="I61" t="s" s="2">
-        <v>16</v>
+        <v>125</v>
       </c>
       <c r="J61" t="s" s="0">
-        <v>161</v>
+        <v>165</v>
       </c>
       <c r="K61" t="s" s="0">
-        <v>155</v>
+        <v>159</v>
       </c>
     </row>
     <row r="62">
       <c r="A62" t="s" s="1">
-        <v>162</v>
+        <v>166</v>
       </c>
       <c r="B62" t="s" s="0">
         <v>12</v>
       </c>
       <c r="C62" t="s" s="1">
-        <v>153</v>
+        <v>157</v>
       </c>
       <c r="D62" t="s" s="0">
-        <v>121</v>
+        <v>124</v>
       </c>
       <c r="E62" t="s" s="0">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="F62" t="s" s="2">
         <v>16</v>
@@ -3144,30 +3156,30 @@
         <v>16</v>
       </c>
       <c r="I62" t="s" s="2">
-        <v>16</v>
+        <v>125</v>
       </c>
       <c r="J62" t="s" s="0">
-        <v>163</v>
+        <v>167</v>
       </c>
       <c r="K62" t="s" s="0">
-        <v>155</v>
+        <v>159</v>
       </c>
     </row>
     <row r="63">
       <c r="A63" t="s" s="1">
-        <v>164</v>
+        <v>168</v>
       </c>
       <c r="B63" t="s" s="0">
         <v>12</v>
       </c>
       <c r="C63" t="s" s="1">
-        <v>153</v>
+        <v>157</v>
       </c>
       <c r="D63" t="s" s="0">
-        <v>121</v>
+        <v>124</v>
       </c>
       <c r="E63" t="s" s="0">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="F63" t="s" s="2">
         <v>16</v>
@@ -3179,30 +3191,30 @@
         <v>16</v>
       </c>
       <c r="I63" t="s" s="2">
-        <v>16</v>
+        <v>125</v>
       </c>
       <c r="J63" t="s" s="0">
-        <v>165</v>
+        <v>169</v>
       </c>
       <c r="K63" t="s" s="0">
-        <v>155</v>
+        <v>159</v>
       </c>
     </row>
     <row r="64">
       <c r="A64" t="s" s="1">
-        <v>166</v>
+        <v>170</v>
       </c>
       <c r="B64" t="s" s="0">
         <v>12</v>
       </c>
       <c r="C64" t="s" s="1">
-        <v>153</v>
+        <v>157</v>
       </c>
       <c r="D64" t="s" s="0">
-        <v>121</v>
+        <v>124</v>
       </c>
       <c r="E64" t="s" s="0">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="F64" t="s" s="2">
         <v>16</v>
@@ -3214,30 +3226,30 @@
         <v>16</v>
       </c>
       <c r="I64" t="s" s="2">
-        <v>16</v>
+        <v>125</v>
       </c>
       <c r="J64" t="s" s="0">
-        <v>167</v>
+        <v>171</v>
       </c>
       <c r="K64" t="s" s="0">
-        <v>155</v>
+        <v>159</v>
       </c>
     </row>
     <row r="65">
       <c r="A65" t="s" s="1">
-        <v>168</v>
+        <v>172</v>
       </c>
       <c r="B65" t="s" s="0">
         <v>12</v>
       </c>
       <c r="C65" t="s" s="1">
-        <v>153</v>
+        <v>157</v>
       </c>
       <c r="D65" t="s" s="0">
-        <v>121</v>
+        <v>124</v>
       </c>
       <c r="E65" t="s" s="0">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="F65" t="s" s="2">
         <v>16</v>
@@ -3249,30 +3261,30 @@
         <v>16</v>
       </c>
       <c r="I65" t="s" s="2">
-        <v>16</v>
+        <v>125</v>
       </c>
       <c r="J65" t="s" s="0">
-        <v>169</v>
+        <v>173</v>
       </c>
       <c r="K65" t="s" s="0">
-        <v>155</v>
+        <v>159</v>
       </c>
     </row>
     <row r="66">
       <c r="A66" t="s" s="1">
-        <v>170</v>
+        <v>174</v>
       </c>
       <c r="B66" t="s" s="0">
         <v>12</v>
       </c>
       <c r="C66" t="s" s="1">
-        <v>153</v>
+        <v>157</v>
       </c>
       <c r="D66" t="s" s="0">
-        <v>121</v>
+        <v>124</v>
       </c>
       <c r="E66" t="s" s="0">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="F66" t="s" s="2">
         <v>16</v>
@@ -3284,30 +3296,30 @@
         <v>16</v>
       </c>
       <c r="I66" t="s" s="2">
-        <v>16</v>
+        <v>125</v>
       </c>
       <c r="J66" t="s" s="0">
-        <v>171</v>
+        <v>175</v>
       </c>
       <c r="K66" t="s" s="0">
-        <v>155</v>
+        <v>159</v>
       </c>
     </row>
     <row r="67">
       <c r="A67" t="s" s="1">
-        <v>172</v>
+        <v>176</v>
       </c>
       <c r="B67" t="s" s="0">
         <v>12</v>
       </c>
       <c r="C67" t="s" s="1">
-        <v>153</v>
+        <v>157</v>
       </c>
       <c r="D67" t="s" s="0">
-        <v>121</v>
+        <v>124</v>
       </c>
       <c r="E67" t="s" s="0">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="F67" t="s" s="2">
         <v>16</v>
@@ -3319,30 +3331,30 @@
         <v>16</v>
       </c>
       <c r="I67" t="s" s="2">
-        <v>16</v>
+        <v>125</v>
       </c>
       <c r="J67" t="s" s="0">
-        <v>173</v>
+        <v>177</v>
       </c>
       <c r="K67" t="s" s="0">
-        <v>155</v>
+        <v>159</v>
       </c>
     </row>
     <row r="68">
       <c r="A68" t="s" s="1">
-        <v>174</v>
+        <v>178</v>
       </c>
       <c r="B68" t="s" s="0">
         <v>12</v>
       </c>
       <c r="C68" t="s" s="1">
-        <v>153</v>
+        <v>157</v>
       </c>
       <c r="D68" t="s" s="0">
-        <v>121</v>
+        <v>124</v>
       </c>
       <c r="E68" t="s" s="0">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="F68" t="s" s="2">
         <v>16</v>
@@ -3354,30 +3366,30 @@
         <v>16</v>
       </c>
       <c r="I68" t="s" s="2">
-        <v>16</v>
+        <v>125</v>
       </c>
       <c r="J68" t="s" s="0">
-        <v>175</v>
+        <v>179</v>
       </c>
       <c r="K68" t="s" s="0">
-        <v>155</v>
+        <v>159</v>
       </c>
     </row>
     <row r="69">
       <c r="A69" t="s" s="1">
-        <v>176</v>
+        <v>180</v>
       </c>
       <c r="B69" t="s" s="0">
         <v>12</v>
       </c>
       <c r="C69" t="s" s="1">
-        <v>153</v>
+        <v>157</v>
       </c>
       <c r="D69" t="s" s="0">
-        <v>121</v>
+        <v>124</v>
       </c>
       <c r="E69" t="s" s="0">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="F69" t="s" s="2">
         <v>16</v>
@@ -3389,30 +3401,30 @@
         <v>16</v>
       </c>
       <c r="I69" t="s" s="2">
-        <v>16</v>
+        <v>125</v>
       </c>
       <c r="J69" t="s" s="0">
-        <v>177</v>
+        <v>181</v>
       </c>
       <c r="K69" t="s" s="0">
-        <v>155</v>
+        <v>159</v>
       </c>
     </row>
     <row r="70">
       <c r="A70" t="s" s="1">
-        <v>178</v>
+        <v>182</v>
       </c>
       <c r="B70" t="s" s="0">
         <v>12</v>
       </c>
       <c r="C70" t="s" s="1">
-        <v>153</v>
+        <v>157</v>
       </c>
       <c r="D70" t="s" s="0">
-        <v>121</v>
+        <v>124</v>
       </c>
       <c r="E70" t="s" s="0">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="F70" t="s" s="2">
         <v>16</v>
@@ -3424,30 +3436,30 @@
         <v>16</v>
       </c>
       <c r="I70" t="s" s="2">
-        <v>16</v>
+        <v>125</v>
       </c>
       <c r="J70" t="s" s="0">
-        <v>179</v>
+        <v>183</v>
       </c>
       <c r="K70" t="s" s="0">
-        <v>155</v>
+        <v>159</v>
       </c>
     </row>
     <row r="71">
       <c r="A71" t="s" s="1">
-        <v>180</v>
+        <v>184</v>
       </c>
       <c r="B71" t="s" s="0">
         <v>12</v>
       </c>
       <c r="C71" t="s" s="1">
-        <v>153</v>
+        <v>157</v>
       </c>
       <c r="D71" t="s" s="0">
-        <v>121</v>
+        <v>124</v>
       </c>
       <c r="E71" t="s" s="0">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="F71" t="s" s="2">
         <v>16</v>
@@ -3459,30 +3471,30 @@
         <v>16</v>
       </c>
       <c r="I71" t="s" s="2">
-        <v>16</v>
+        <v>125</v>
       </c>
       <c r="J71" t="s" s="0">
-        <v>181</v>
+        <v>185</v>
       </c>
       <c r="K71" t="s" s="0">
-        <v>155</v>
+        <v>159</v>
       </c>
     </row>
     <row r="72">
       <c r="A72" t="s" s="1">
-        <v>182</v>
+        <v>186</v>
       </c>
       <c r="B72" t="s" s="0">
         <v>12</v>
       </c>
       <c r="C72" t="s" s="1">
-        <v>153</v>
+        <v>157</v>
       </c>
       <c r="D72" t="s" s="0">
-        <v>121</v>
+        <v>124</v>
       </c>
       <c r="E72" t="s" s="0">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="F72" t="s" s="2">
         <v>16</v>
@@ -3494,30 +3506,30 @@
         <v>16</v>
       </c>
       <c r="I72" t="s" s="2">
-        <v>16</v>
+        <v>125</v>
       </c>
       <c r="J72" t="s" s="0">
-        <v>183</v>
+        <v>187</v>
       </c>
       <c r="K72" t="s" s="0">
-        <v>155</v>
+        <v>159</v>
       </c>
     </row>
     <row r="73">
       <c r="A73" t="s" s="1">
-        <v>184</v>
+        <v>188</v>
       </c>
       <c r="B73" t="s" s="0">
         <v>12</v>
       </c>
       <c r="C73" t="s" s="1">
-        <v>153</v>
+        <v>157</v>
       </c>
       <c r="D73" t="s" s="0">
-        <v>121</v>
+        <v>124</v>
       </c>
       <c r="E73" t="s" s="0">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="F73" t="s" s="2">
         <v>16</v>
@@ -3529,30 +3541,30 @@
         <v>16</v>
       </c>
       <c r="I73" t="s" s="2">
-        <v>16</v>
+        <v>125</v>
       </c>
       <c r="J73" t="s" s="0">
-        <v>185</v>
+        <v>189</v>
       </c>
       <c r="K73" t="s" s="0">
-        <v>155</v>
+        <v>159</v>
       </c>
     </row>
     <row r="74">
       <c r="A74" t="s" s="1">
-        <v>186</v>
+        <v>190</v>
       </c>
       <c r="B74" t="s" s="0">
         <v>12</v>
       </c>
       <c r="C74" t="s" s="1">
-        <v>153</v>
+        <v>157</v>
       </c>
       <c r="D74" t="s" s="0">
-        <v>121</v>
+        <v>124</v>
       </c>
       <c r="E74" t="s" s="0">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="F74" t="s" s="2">
         <v>16</v>
@@ -3564,30 +3576,30 @@
         <v>16</v>
       </c>
       <c r="I74" t="s" s="2">
-        <v>16</v>
+        <v>125</v>
       </c>
       <c r="J74" t="s" s="0">
-        <v>187</v>
+        <v>191</v>
       </c>
       <c r="K74" t="s" s="0">
-        <v>155</v>
+        <v>159</v>
       </c>
     </row>
     <row r="75">
       <c r="A75" t="s" s="1">
-        <v>188</v>
+        <v>192</v>
       </c>
       <c r="B75" t="s" s="0">
         <v>12</v>
       </c>
       <c r="C75" t="s" s="1">
-        <v>153</v>
+        <v>157</v>
       </c>
       <c r="D75" t="s" s="0">
-        <v>121</v>
+        <v>124</v>
       </c>
       <c r="E75" t="s" s="0">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="F75" t="s" s="2">
         <v>16</v>
@@ -3599,30 +3611,30 @@
         <v>16</v>
       </c>
       <c r="I75" t="s" s="2">
-        <v>16</v>
+        <v>125</v>
       </c>
       <c r="J75" t="s" s="0">
-        <v>189</v>
+        <v>193</v>
       </c>
       <c r="K75" t="s" s="0">
-        <v>155</v>
+        <v>159</v>
       </c>
     </row>
     <row r="76">
       <c r="A76" t="s" s="1">
-        <v>190</v>
+        <v>194</v>
       </c>
       <c r="B76" t="s" s="0">
         <v>12</v>
       </c>
       <c r="C76" t="s" s="1">
-        <v>153</v>
+        <v>157</v>
       </c>
       <c r="D76" t="s" s="0">
-        <v>121</v>
+        <v>124</v>
       </c>
       <c r="E76" t="s" s="0">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="F76" t="s" s="2">
         <v>16</v>
@@ -3634,30 +3646,30 @@
         <v>16</v>
       </c>
       <c r="I76" t="s" s="2">
-        <v>16</v>
+        <v>125</v>
       </c>
       <c r="J76" t="s" s="0">
-        <v>191</v>
+        <v>195</v>
       </c>
       <c r="K76" t="s" s="0">
-        <v>155</v>
+        <v>159</v>
       </c>
     </row>
     <row r="77">
       <c r="A77" t="s" s="1">
-        <v>192</v>
+        <v>196</v>
       </c>
       <c r="B77" t="s" s="0">
         <v>12</v>
       </c>
       <c r="C77" t="s" s="1">
-        <v>153</v>
+        <v>157</v>
       </c>
       <c r="D77" t="s" s="0">
-        <v>121</v>
+        <v>124</v>
       </c>
       <c r="E77" t="s" s="0">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="F77" t="s" s="2">
         <v>16</v>
@@ -3669,30 +3681,30 @@
         <v>16</v>
       </c>
       <c r="I77" t="s" s="2">
-        <v>16</v>
+        <v>125</v>
       </c>
       <c r="J77" t="s" s="0">
-        <v>193</v>
+        <v>197</v>
       </c>
       <c r="K77" t="s" s="0">
-        <v>155</v>
+        <v>159</v>
       </c>
     </row>
     <row r="78">
       <c r="A78" t="s" s="1">
-        <v>194</v>
+        <v>198</v>
       </c>
       <c r="B78" t="s" s="0">
         <v>12</v>
       </c>
       <c r="C78" t="s" s="1">
-        <v>153</v>
+        <v>157</v>
       </c>
       <c r="D78" t="s" s="0">
-        <v>121</v>
+        <v>124</v>
       </c>
       <c r="E78" t="s" s="0">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="F78" t="s" s="2">
         <v>16</v>
@@ -3704,30 +3716,30 @@
         <v>16</v>
       </c>
       <c r="I78" t="s" s="2">
-        <v>16</v>
+        <v>125</v>
       </c>
       <c r="J78" t="s" s="0">
-        <v>195</v>
+        <v>199</v>
       </c>
       <c r="K78" t="s" s="0">
-        <v>155</v>
+        <v>159</v>
       </c>
     </row>
     <row r="79">
       <c r="A79" t="s" s="1">
-        <v>196</v>
+        <v>200</v>
       </c>
       <c r="B79" t="s" s="0">
         <v>12</v>
       </c>
       <c r="C79" t="s" s="1">
-        <v>153</v>
+        <v>157</v>
       </c>
       <c r="D79" t="s" s="0">
-        <v>121</v>
+        <v>124</v>
       </c>
       <c r="E79" t="s" s="0">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="F79" t="s" s="2">
         <v>16</v>
@@ -3739,30 +3751,30 @@
         <v>16</v>
       </c>
       <c r="I79" t="s" s="2">
-        <v>16</v>
+        <v>125</v>
       </c>
       <c r="J79" t="s" s="0">
-        <v>197</v>
+        <v>201</v>
       </c>
       <c r="K79" t="s" s="0">
-        <v>155</v>
+        <v>159</v>
       </c>
     </row>
     <row r="80">
       <c r="A80" t="s" s="1">
-        <v>198</v>
+        <v>202</v>
       </c>
       <c r="B80" t="s" s="0">
         <v>12</v>
       </c>
       <c r="C80" t="s" s="1">
-        <v>153</v>
+        <v>157</v>
       </c>
       <c r="D80" t="s" s="0">
-        <v>121</v>
+        <v>124</v>
       </c>
       <c r="E80" t="s" s="0">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="F80" t="s" s="2">
         <v>16</v>
@@ -3774,30 +3786,30 @@
         <v>16</v>
       </c>
       <c r="I80" t="s" s="2">
-        <v>16</v>
+        <v>125</v>
       </c>
       <c r="J80" t="s" s="0">
-        <v>199</v>
+        <v>203</v>
       </c>
       <c r="K80" t="s" s="0">
-        <v>155</v>
+        <v>159</v>
       </c>
     </row>
     <row r="81">
       <c r="A81" t="s" s="1">
-        <v>200</v>
+        <v>204</v>
       </c>
       <c r="B81" t="s" s="0">
         <v>12</v>
       </c>
       <c r="C81" t="s" s="1">
-        <v>153</v>
+        <v>157</v>
       </c>
       <c r="D81" t="s" s="0">
-        <v>121</v>
+        <v>124</v>
       </c>
       <c r="E81" t="s" s="0">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="F81" t="s" s="2">
         <v>16</v>
@@ -3809,30 +3821,30 @@
         <v>16</v>
       </c>
       <c r="I81" t="s" s="2">
-        <v>16</v>
+        <v>125</v>
       </c>
       <c r="J81" t="s" s="0">
-        <v>201</v>
+        <v>205</v>
       </c>
       <c r="K81" t="s" s="0">
-        <v>155</v>
+        <v>159</v>
       </c>
     </row>
     <row r="82">
       <c r="A82" t="s" s="1">
-        <v>202</v>
+        <v>206</v>
       </c>
       <c r="B82" t="s" s="0">
         <v>12</v>
       </c>
       <c r="C82" t="s" s="1">
-        <v>153</v>
+        <v>157</v>
       </c>
       <c r="D82" t="s" s="0">
-        <v>121</v>
+        <v>124</v>
       </c>
       <c r="E82" t="s" s="0">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="F82" t="s" s="2">
         <v>16</v>
@@ -3844,30 +3856,30 @@
         <v>16</v>
       </c>
       <c r="I82" t="s" s="2">
-        <v>16</v>
+        <v>125</v>
       </c>
       <c r="J82" t="s" s="0">
-        <v>203</v>
+        <v>207</v>
       </c>
       <c r="K82" t="s" s="0">
-        <v>155</v>
+        <v>159</v>
       </c>
     </row>
     <row r="83">
       <c r="A83" t="s" s="1">
-        <v>204</v>
+        <v>208</v>
       </c>
       <c r="B83" t="s" s="0">
         <v>12</v>
       </c>
       <c r="C83" t="s" s="1">
-        <v>153</v>
+        <v>157</v>
       </c>
       <c r="D83" t="s" s="0">
-        <v>121</v>
+        <v>124</v>
       </c>
       <c r="E83" t="s" s="0">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="F83" t="s" s="2">
         <v>16</v>
@@ -3879,30 +3891,30 @@
         <v>16</v>
       </c>
       <c r="I83" t="s" s="2">
-        <v>16</v>
+        <v>125</v>
       </c>
       <c r="J83" t="s" s="0">
-        <v>205</v>
+        <v>209</v>
       </c>
       <c r="K83" t="s" s="0">
-        <v>155</v>
+        <v>159</v>
       </c>
     </row>
     <row r="84">
       <c r="A84" t="s" s="1">
-        <v>206</v>
+        <v>210</v>
       </c>
       <c r="B84" t="s" s="0">
         <v>12</v>
       </c>
       <c r="C84" t="s" s="1">
-        <v>153</v>
+        <v>157</v>
       </c>
       <c r="D84" t="s" s="0">
-        <v>121</v>
+        <v>124</v>
       </c>
       <c r="E84" t="s" s="0">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="F84" t="s" s="2">
         <v>16</v>
@@ -3914,30 +3926,30 @@
         <v>16</v>
       </c>
       <c r="I84" t="s" s="2">
-        <v>16</v>
+        <v>125</v>
       </c>
       <c r="J84" t="s" s="0">
-        <v>207</v>
+        <v>211</v>
       </c>
       <c r="K84" t="s" s="0">
-        <v>155</v>
+        <v>159</v>
       </c>
     </row>
     <row r="85">
       <c r="A85" t="s" s="1">
-        <v>208</v>
+        <v>212</v>
       </c>
       <c r="B85" t="s" s="0">
         <v>12</v>
       </c>
       <c r="C85" t="s" s="1">
-        <v>153</v>
+        <v>157</v>
       </c>
       <c r="D85" t="s" s="0">
-        <v>121</v>
+        <v>124</v>
       </c>
       <c r="E85" t="s" s="0">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="F85" t="s" s="2">
         <v>16</v>
@@ -3949,30 +3961,30 @@
         <v>16</v>
       </c>
       <c r="I85" t="s" s="2">
-        <v>16</v>
+        <v>125</v>
       </c>
       <c r="J85" t="s" s="0">
-        <v>209</v>
+        <v>213</v>
       </c>
       <c r="K85" t="s" s="0">
-        <v>155</v>
+        <v>159</v>
       </c>
     </row>
     <row r="86">
       <c r="A86" t="s" s="1">
-        <v>210</v>
+        <v>214</v>
       </c>
       <c r="B86" t="s" s="0">
         <v>12</v>
       </c>
       <c r="C86" t="s" s="1">
-        <v>153</v>
+        <v>157</v>
       </c>
       <c r="D86" t="s" s="0">
-        <v>121</v>
+        <v>124</v>
       </c>
       <c r="E86" t="s" s="0">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="F86" t="s" s="2">
         <v>16</v>
@@ -3984,30 +3996,30 @@
         <v>16</v>
       </c>
       <c r="I86" t="s" s="2">
-        <v>16</v>
+        <v>125</v>
       </c>
       <c r="J86" t="s" s="0">
-        <v>211</v>
+        <v>215</v>
       </c>
       <c r="K86" t="s" s="0">
-        <v>155</v>
+        <v>159</v>
       </c>
     </row>
     <row r="87">
       <c r="A87" t="s" s="1">
-        <v>212</v>
+        <v>216</v>
       </c>
       <c r="B87" t="s" s="0">
         <v>12</v>
       </c>
       <c r="C87" t="s" s="1">
-        <v>153</v>
+        <v>157</v>
       </c>
       <c r="D87" t="s" s="0">
-        <v>121</v>
+        <v>124</v>
       </c>
       <c r="E87" t="s" s="0">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="F87" t="s" s="2">
         <v>16</v>
@@ -4019,30 +4031,30 @@
         <v>16</v>
       </c>
       <c r="I87" t="s" s="2">
-        <v>16</v>
+        <v>125</v>
       </c>
       <c r="J87" t="s" s="0">
-        <v>213</v>
+        <v>217</v>
       </c>
       <c r="K87" t="s" s="0">
-        <v>155</v>
+        <v>159</v>
       </c>
     </row>
     <row r="88">
       <c r="A88" t="s" s="1">
-        <v>214</v>
+        <v>218</v>
       </c>
       <c r="B88" t="s" s="0">
         <v>12</v>
       </c>
       <c r="C88" t="s" s="1">
-        <v>153</v>
+        <v>157</v>
       </c>
       <c r="D88" t="s" s="0">
-        <v>121</v>
+        <v>124</v>
       </c>
       <c r="E88" t="s" s="0">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="F88" t="s" s="2">
         <v>16</v>
@@ -4054,30 +4066,30 @@
         <v>16</v>
       </c>
       <c r="I88" t="s" s="2">
-        <v>16</v>
+        <v>125</v>
       </c>
       <c r="J88" t="s" s="0">
-        <v>215</v>
+        <v>219</v>
       </c>
       <c r="K88" t="s" s="0">
-        <v>155</v>
+        <v>159</v>
       </c>
     </row>
     <row r="89">
       <c r="A89" t="s" s="1">
-        <v>216</v>
+        <v>220</v>
       </c>
       <c r="B89" t="s" s="0">
         <v>12</v>
       </c>
       <c r="C89" t="s" s="1">
-        <v>153</v>
+        <v>157</v>
       </c>
       <c r="D89" t="s" s="0">
-        <v>121</v>
+        <v>124</v>
       </c>
       <c r="E89" t="s" s="0">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="F89" t="s" s="2">
         <v>16</v>
@@ -4089,30 +4101,30 @@
         <v>16</v>
       </c>
       <c r="I89" t="s" s="2">
-        <v>16</v>
+        <v>125</v>
       </c>
       <c r="J89" t="s" s="0">
-        <v>217</v>
+        <v>221</v>
       </c>
       <c r="K89" t="s" s="0">
-        <v>155</v>
+        <v>159</v>
       </c>
     </row>
     <row r="90">
       <c r="A90" t="s" s="1">
-        <v>218</v>
+        <v>222</v>
       </c>
       <c r="B90" t="s" s="0">
         <v>12</v>
       </c>
       <c r="C90" t="s" s="1">
-        <v>153</v>
+        <v>157</v>
       </c>
       <c r="D90" t="s" s="0">
-        <v>121</v>
+        <v>124</v>
       </c>
       <c r="E90" t="s" s="0">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="F90" t="s" s="2">
         <v>16</v>
@@ -4124,30 +4136,30 @@
         <v>16</v>
       </c>
       <c r="I90" t="s" s="2">
-        <v>16</v>
+        <v>125</v>
       </c>
       <c r="J90" t="s" s="0">
-        <v>219</v>
+        <v>223</v>
       </c>
       <c r="K90" t="s" s="0">
-        <v>155</v>
+        <v>159</v>
       </c>
     </row>
     <row r="91">
       <c r="A91" t="s" s="1">
-        <v>220</v>
+        <v>224</v>
       </c>
       <c r="B91" t="s" s="0">
         <v>12</v>
       </c>
       <c r="C91" t="s" s="1">
-        <v>153</v>
+        <v>157</v>
       </c>
       <c r="D91" t="s" s="0">
-        <v>121</v>
+        <v>124</v>
       </c>
       <c r="E91" t="s" s="0">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="F91" t="s" s="2">
         <v>16</v>
@@ -4159,30 +4171,30 @@
         <v>16</v>
       </c>
       <c r="I91" t="s" s="2">
-        <v>16</v>
+        <v>125</v>
       </c>
       <c r="J91" t="s" s="0">
-        <v>221</v>
+        <v>225</v>
       </c>
       <c r="K91" t="s" s="0">
-        <v>155</v>
+        <v>159</v>
       </c>
     </row>
     <row r="92">
       <c r="A92" t="s" s="1">
-        <v>222</v>
+        <v>226</v>
       </c>
       <c r="B92" t="s" s="0">
         <v>12</v>
       </c>
       <c r="C92" t="s" s="1">
-        <v>153</v>
+        <v>157</v>
       </c>
       <c r="D92" t="s" s="0">
-        <v>121</v>
+        <v>124</v>
       </c>
       <c r="E92" t="s" s="0">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="F92" t="s" s="2">
         <v>16</v>
@@ -4194,30 +4206,30 @@
         <v>16</v>
       </c>
       <c r="I92" t="s" s="2">
-        <v>16</v>
+        <v>125</v>
       </c>
       <c r="J92" t="s" s="0">
-        <v>223</v>
+        <v>227</v>
       </c>
       <c r="K92" t="s" s="0">
-        <v>155</v>
+        <v>159</v>
       </c>
     </row>
     <row r="93">
       <c r="A93" t="s" s="1">
-        <v>224</v>
+        <v>228</v>
       </c>
       <c r="B93" t="s" s="0">
         <v>12</v>
       </c>
       <c r="C93" t="s" s="1">
-        <v>153</v>
+        <v>157</v>
       </c>
       <c r="D93" t="s" s="0">
-        <v>121</v>
+        <v>124</v>
       </c>
       <c r="E93" t="s" s="0">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="F93" t="s" s="2">
         <v>16</v>
@@ -4229,30 +4241,30 @@
         <v>16</v>
       </c>
       <c r="I93" t="s" s="2">
-        <v>16</v>
+        <v>125</v>
       </c>
       <c r="J93" t="s" s="0">
-        <v>225</v>
+        <v>229</v>
       </c>
       <c r="K93" t="s" s="0">
-        <v>155</v>
+        <v>159</v>
       </c>
     </row>
     <row r="94">
       <c r="A94" t="s" s="1">
-        <v>226</v>
+        <v>230</v>
       </c>
       <c r="B94" t="s" s="0">
         <v>12</v>
       </c>
       <c r="C94" t="s" s="1">
-        <v>153</v>
+        <v>157</v>
       </c>
       <c r="D94" t="s" s="0">
-        <v>121</v>
+        <v>124</v>
       </c>
       <c r="E94" t="s" s="0">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="F94" t="s" s="2">
         <v>16</v>
@@ -4264,30 +4276,30 @@
         <v>16</v>
       </c>
       <c r="I94" t="s" s="2">
-        <v>16</v>
+        <v>125</v>
       </c>
       <c r="J94" t="s" s="0">
-        <v>227</v>
+        <v>231</v>
       </c>
       <c r="K94" t="s" s="0">
-        <v>155</v>
+        <v>159</v>
       </c>
     </row>
     <row r="95">
       <c r="A95" t="s" s="1">
-        <v>228</v>
+        <v>232</v>
       </c>
       <c r="B95" t="s" s="0">
         <v>12</v>
       </c>
       <c r="C95" t="s" s="1">
-        <v>153</v>
+        <v>157</v>
       </c>
       <c r="D95" t="s" s="0">
-        <v>121</v>
+        <v>124</v>
       </c>
       <c r="E95" t="s" s="0">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="F95" t="s" s="2">
         <v>16</v>
@@ -4299,30 +4311,30 @@
         <v>16</v>
       </c>
       <c r="I95" t="s" s="2">
-        <v>16</v>
+        <v>125</v>
       </c>
       <c r="J95" t="s" s="0">
-        <v>229</v>
+        <v>233</v>
       </c>
       <c r="K95" t="s" s="0">
-        <v>155</v>
+        <v>159</v>
       </c>
     </row>
     <row r="96">
       <c r="A96" t="s" s="1">
-        <v>230</v>
+        <v>234</v>
       </c>
       <c r="B96" t="s" s="0">
         <v>12</v>
       </c>
       <c r="C96" t="s" s="1">
-        <v>153</v>
+        <v>157</v>
       </c>
       <c r="D96" t="s" s="0">
-        <v>121</v>
+        <v>124</v>
       </c>
       <c r="E96" t="s" s="0">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="F96" t="s" s="2">
         <v>16</v>
@@ -4334,30 +4346,30 @@
         <v>16</v>
       </c>
       <c r="I96" t="s" s="2">
-        <v>16</v>
+        <v>125</v>
       </c>
       <c r="J96" t="s" s="0">
-        <v>231</v>
+        <v>235</v>
       </c>
       <c r="K96" t="s" s="0">
-        <v>155</v>
+        <v>159</v>
       </c>
     </row>
     <row r="97">
       <c r="A97" t="s" s="1">
-        <v>232</v>
+        <v>236</v>
       </c>
       <c r="B97" t="s" s="0">
         <v>12</v>
       </c>
       <c r="C97" t="s" s="1">
-        <v>153</v>
+        <v>157</v>
       </c>
       <c r="D97" t="s" s="0">
-        <v>121</v>
+        <v>124</v>
       </c>
       <c r="E97" t="s" s="0">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="F97" t="s" s="2">
         <v>16</v>
@@ -4369,30 +4381,30 @@
         <v>16</v>
       </c>
       <c r="I97" t="s" s="2">
-        <v>16</v>
+        <v>125</v>
       </c>
       <c r="J97" t="s" s="0">
-        <v>233</v>
+        <v>237</v>
       </c>
       <c r="K97" t="s" s="0">
-        <v>155</v>
+        <v>159</v>
       </c>
     </row>
     <row r="98">
       <c r="A98" t="s" s="1">
-        <v>234</v>
+        <v>238</v>
       </c>
       <c r="B98" t="s" s="0">
         <v>12</v>
       </c>
       <c r="C98" t="s" s="1">
-        <v>153</v>
+        <v>157</v>
       </c>
       <c r="D98" t="s" s="0">
-        <v>121</v>
+        <v>124</v>
       </c>
       <c r="E98" t="s" s="0">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="F98" t="s" s="2">
         <v>16</v>
@@ -4404,30 +4416,30 @@
         <v>16</v>
       </c>
       <c r="I98" t="s" s="2">
-        <v>16</v>
+        <v>125</v>
       </c>
       <c r="J98" t="s" s="0">
-        <v>235</v>
+        <v>239</v>
       </c>
       <c r="K98" t="s" s="0">
-        <v>155</v>
+        <v>159</v>
       </c>
     </row>
     <row r="99">
       <c r="A99" t="s" s="1">
-        <v>236</v>
+        <v>240</v>
       </c>
       <c r="B99" t="s" s="0">
         <v>12</v>
       </c>
       <c r="C99" t="s" s="1">
-        <v>153</v>
+        <v>157</v>
       </c>
       <c r="D99" t="s" s="0">
-        <v>121</v>
+        <v>124</v>
       </c>
       <c r="E99" t="s" s="0">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="F99" t="s" s="2">
         <v>16</v>
@@ -4439,30 +4451,30 @@
         <v>16</v>
       </c>
       <c r="I99" t="s" s="2">
-        <v>16</v>
+        <v>125</v>
       </c>
       <c r="J99" t="s" s="0">
-        <v>237</v>
+        <v>241</v>
       </c>
       <c r="K99" t="s" s="0">
-        <v>155</v>
+        <v>159</v>
       </c>
     </row>
     <row r="100">
       <c r="A100" t="s" s="1">
-        <v>238</v>
+        <v>242</v>
       </c>
       <c r="B100" t="s" s="0">
         <v>12</v>
       </c>
       <c r="C100" t="s" s="1">
-        <v>153</v>
+        <v>157</v>
       </c>
       <c r="D100" t="s" s="0">
-        <v>121</v>
+        <v>124</v>
       </c>
       <c r="E100" t="s" s="0">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="F100" t="s" s="2">
         <v>16</v>
@@ -4474,30 +4486,30 @@
         <v>16</v>
       </c>
       <c r="I100" t="s" s="2">
-        <v>16</v>
+        <v>125</v>
       </c>
       <c r="J100" t="s" s="0">
-        <v>239</v>
+        <v>243</v>
       </c>
       <c r="K100" t="s" s="0">
-        <v>155</v>
+        <v>159</v>
       </c>
     </row>
     <row r="101">
       <c r="A101" t="s" s="1">
-        <v>240</v>
+        <v>244</v>
       </c>
       <c r="B101" t="s" s="0">
         <v>12</v>
       </c>
       <c r="C101" t="s" s="1">
-        <v>153</v>
+        <v>157</v>
       </c>
       <c r="D101" t="s" s="0">
-        <v>121</v>
+        <v>124</v>
       </c>
       <c r="E101" t="s" s="0">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="F101" t="s" s="2">
         <v>16</v>
@@ -4509,30 +4521,30 @@
         <v>16</v>
       </c>
       <c r="I101" t="s" s="2">
-        <v>16</v>
+        <v>125</v>
       </c>
       <c r="J101" t="s" s="0">
-        <v>241</v>
+        <v>245</v>
       </c>
       <c r="K101" t="s" s="0">
-        <v>155</v>
+        <v>159</v>
       </c>
     </row>
     <row r="102">
       <c r="A102" t="s" s="1">
-        <v>242</v>
+        <v>246</v>
       </c>
       <c r="B102" t="s" s="0">
         <v>12</v>
       </c>
       <c r="C102" t="s" s="1">
-        <v>153</v>
+        <v>157</v>
       </c>
       <c r="D102" t="s" s="0">
-        <v>121</v>
+        <v>124</v>
       </c>
       <c r="E102" t="s" s="0">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="F102" t="s" s="2">
         <v>16</v>
@@ -4544,30 +4556,30 @@
         <v>16</v>
       </c>
       <c r="I102" t="s" s="2">
-        <v>16</v>
+        <v>125</v>
       </c>
       <c r="J102" t="s" s="0">
-        <v>243</v>
+        <v>247</v>
       </c>
       <c r="K102" t="s" s="0">
-        <v>155</v>
+        <v>159</v>
       </c>
     </row>
     <row r="103">
       <c r="A103" t="s" s="1">
-        <v>244</v>
+        <v>248</v>
       </c>
       <c r="B103" t="s" s="0">
         <v>12</v>
       </c>
       <c r="C103" t="s" s="1">
-        <v>153</v>
+        <v>157</v>
       </c>
       <c r="D103" t="s" s="0">
-        <v>121</v>
+        <v>124</v>
       </c>
       <c r="E103" t="s" s="0">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="F103" t="s" s="2">
         <v>16</v>
@@ -4579,30 +4591,30 @@
         <v>16</v>
       </c>
       <c r="I103" t="s" s="2">
-        <v>16</v>
+        <v>125</v>
       </c>
       <c r="J103" t="s" s="0">
-        <v>245</v>
+        <v>249</v>
       </c>
       <c r="K103" t="s" s="0">
-        <v>155</v>
+        <v>159</v>
       </c>
     </row>
     <row r="104">
       <c r="A104" t="s" s="1">
-        <v>246</v>
+        <v>250</v>
       </c>
       <c r="B104" t="s" s="0">
         <v>12</v>
       </c>
       <c r="C104" t="s" s="1">
-        <v>153</v>
+        <v>157</v>
       </c>
       <c r="D104" t="s" s="0">
-        <v>121</v>
+        <v>124</v>
       </c>
       <c r="E104" t="s" s="0">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="F104" t="s" s="2">
         <v>16</v>
@@ -4614,30 +4626,30 @@
         <v>16</v>
       </c>
       <c r="I104" t="s" s="2">
-        <v>16</v>
+        <v>125</v>
       </c>
       <c r="J104" t="s" s="0">
-        <v>247</v>
+        <v>251</v>
       </c>
       <c r="K104" t="s" s="0">
-        <v>155</v>
+        <v>159</v>
       </c>
     </row>
     <row r="105">
       <c r="A105" t="s" s="1">
-        <v>248</v>
+        <v>252</v>
       </c>
       <c r="B105" t="s" s="0">
         <v>12</v>
       </c>
       <c r="C105" t="s" s="1">
-        <v>153</v>
+        <v>157</v>
       </c>
       <c r="D105" t="s" s="0">
-        <v>121</v>
+        <v>124</v>
       </c>
       <c r="E105" t="s" s="0">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="F105" t="s" s="2">
         <v>16</v>
@@ -4649,13 +4661,13 @@
         <v>16</v>
       </c>
       <c r="I105" t="s" s="2">
-        <v>16</v>
+        <v>125</v>
       </c>
       <c r="J105" t="s" s="0">
-        <v>249</v>
+        <v>253</v>
       </c>
       <c r="K105" t="s" s="0">
-        <v>155</v>
+        <v>159</v>
       </c>
     </row>
   </sheetData>
@@ -4893,77 +4905,77 @@
     </row>
     <row r="2">
       <c r="A2" t="s" s="0">
-        <v>250</v>
+        <v>254</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="s" s="0">
-        <v>251</v>
+        <v>255</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="s" s="0">
-        <v>252</v>
+        <v>256</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="s" s="0">
-        <v>253</v>
+        <v>257</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="s" s="0">
-        <v>254</v>
+        <v>258</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="s" s="0">
-        <v>255</v>
+        <v>259</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="s" s="0">
-        <v>256</v>
+        <v>260</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="s" s="0">
-        <v>257</v>
+        <v>261</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="s" s="0">
-        <v>258</v>
+        <v>262</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="s" s="0">
-        <v>259</v>
+        <v>263</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="s" s="0">
-        <v>260</v>
+        <v>264</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="s" s="0">
-        <v>261</v>
+        <v>265</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="s" s="0">
-        <v>262</v>
+        <v>266</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="s" s="0">
-        <v>263</v>
+        <v>267</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="s" s="0">
-        <v>264</v>
+        <v>268</v>
       </c>
     </row>
     <row r="17">
@@ -4973,132 +4985,132 @@
     </row>
     <row r="18">
       <c r="A18" t="s" s="0">
-        <v>265</v>
+        <v>269</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="s" s="0">
-        <v>266</v>
+        <v>270</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="s" s="0">
-        <v>267</v>
+        <v>271</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="s" s="0">
-        <v>268</v>
+        <v>272</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="s" s="0">
-        <v>269</v>
+        <v>273</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="s" s="0">
-        <v>270</v>
+        <v>274</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="s" s="0">
-        <v>271</v>
+        <v>275</v>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="s" s="0">
-        <v>272</v>
+        <v>276</v>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="s" s="0">
-        <v>273</v>
+        <v>277</v>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="s" s="0">
-        <v>274</v>
+        <v>278</v>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="s" s="0">
-        <v>275</v>
+        <v>279</v>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="s" s="0">
-        <v>276</v>
+        <v>280</v>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="s" s="0">
-        <v>277</v>
+        <v>281</v>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="s" s="0">
-        <v>278</v>
+        <v>282</v>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="s" s="0">
-        <v>279</v>
+        <v>283</v>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="s" s="0">
-        <v>280</v>
+        <v>284</v>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="s" s="0">
-        <v>281</v>
+        <v>285</v>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="s" s="0">
-        <v>282</v>
+        <v>286</v>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="s" s="0">
-        <v>283</v>
+        <v>287</v>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="s" s="0">
-        <v>284</v>
+        <v>288</v>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="s" s="0">
-        <v>285</v>
+        <v>289</v>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="s" s="0">
-        <v>286</v>
+        <v>290</v>
       </c>
     </row>
     <row r="40">
       <c r="A40" t="s" s="0">
-        <v>287</v>
+        <v>291</v>
       </c>
     </row>
     <row r="41">
       <c r="A41" t="s" s="0">
-        <v>288</v>
+        <v>292</v>
       </c>
     </row>
     <row r="42">
       <c r="A42" t="s" s="0">
-        <v>289</v>
+        <v>293</v>
       </c>
     </row>
     <row r="43">
       <c r="A43" t="s" s="0">
-        <v>290</v>
+        <v>294</v>
       </c>
     </row>
   </sheetData>

</xml_diff>